<commit_message>
rewrite the touch function
</commit_message>
<xml_diff>
--- a/AT32 FOR LVGL/app/project/MDK_V5/AT32F403AVGT7_WorkBench_analysis.xlsx
+++ b/AT32 FOR LVGL/app/project/MDK_V5/AT32F403AVGT7_WorkBench_analysis.xlsx
@@ -15,12 +15,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="72">
   <si>
     <t>AT32F403AVGT7_WorkBench</t>
   </si>
   <si>
-    <t>lto-llvm-92863b.o</t>
+    <t>lto-llvm-b5a238.o</t>
   </si>
   <si>
     <t>startup_at32f403a_407.o</t>
@@ -53,9 +53,6 @@
     <t>fopen.o</t>
   </si>
   <si>
-    <t>_printf_intcommon.o</t>
-  </si>
-  <si>
     <t>rt_memcpy_v6.o</t>
   </si>
   <si>
@@ -65,15 +62,9 @@
     <t>strcmpv7em.o</t>
   </si>
   <si>
-    <t>_printf_dec.o</t>
-  </si>
-  <si>
     <t>llsdiv.o</t>
   </si>
   <si>
-    <t>__printf.o</t>
-  </si>
-  <si>
     <t>rt_memcpy_w.o</t>
   </si>
   <si>
@@ -122,18 +113,12 @@
     <t>defsig_general.o</t>
   </si>
   <si>
-    <t>_printf_char_common.o</t>
-  </si>
-  <si>
     <t>puts.o</t>
   </si>
   <si>
     <t>init_aeabi.o</t>
   </si>
   <si>
-    <t>_printf_char_file.o</t>
-  </si>
-  <si>
     <t>systick_wrapper_gnu.o</t>
   </si>
   <si>
@@ -152,9 +137,6 @@
     <t>__scatter_copy.o</t>
   </si>
   <si>
-    <t>noretval__2printf.o</t>
-  </si>
-  <si>
     <t>libinit2.o</t>
   </si>
   <si>
@@ -194,9 +176,6 @@
     <t>rt_errno_addr_intlibspace.o</t>
   </si>
   <si>
-    <t>ferror.o</t>
-  </si>
-  <si>
     <t>__main.o</t>
   </si>
   <si>
@@ -206,16 +185,10 @@
     <t>heapauxi.o</t>
   </si>
   <si>
-    <t>_printf_u.o</t>
-  </si>
-  <si>
     <t>__rtentry4.o</t>
   </si>
   <si>
     <t>hguard.o</t>
-  </si>
-  <si>
-    <t>_printf_percent_end.o</t>
   </si>
   <si>
     <t>use_no_semi.o</t>
@@ -347,11 +320,11 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>ram_percent!$A$3:$A$73</c:f>
+              <c:f>ram_percent!$A$3:$A$64</c:f>
               <c:strCache>
-                <c:ptCount val="71"/>
+                <c:ptCount val="62"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-92863b.o</c:v>
+                  <c:v>lto-llvm-b5a238.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>startup_at32f403a_407.o</c:v>
@@ -365,7 +338,7 @@
                 <c:pt idx="4">
                   <c:v>libspace.o</c:v>
                 </c:pt>
-                <c:pt idx="70">
+                <c:pt idx="61">
                   <c:v>Totals</c:v>
                 </c:pt>
               </c:strCache>
@@ -373,26 +346,26 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>ram_percent!$B$3:$B$73</c:f>
+              <c:f>ram_percent!$B$3:$B$64</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="71"/>
+                <c:ptCount val="62"/>
                 <c:pt idx="0">
-                  <c:v>98.32932281494141</c:v>
+                  <c:v>98.3292236328125</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.137482881546021</c:v>
+                  <c:v>1.137550234794617</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.2665975391864777</c:v>
+                  <c:v>0.2666133344173431</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.1955048739910126</c:v>
+                  <c:v>0.1955164521932602</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.07109268009662628</c:v>
-                </c:pt>
-                <c:pt idx="70">
+                  <c:v>0.07109688967466354</c:v>
+                </c:pt>
+                <c:pt idx="61">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -460,11 +433,11 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>flash_percent!$A$3:$A$73</c:f>
+              <c:f>flash_percent!$A$3:$A$64</c:f>
               <c:strCache>
-                <c:ptCount val="71"/>
+                <c:ptCount val="62"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-92863b.o</c:v>
+                  <c:v>lto-llvm-b5a238.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>c_w.l</c:v>
@@ -491,189 +464,162 @@
                   <c:v>fopen.o</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>_printf_intcommon.o</c:v>
+                  <c:v>rt_memcpy_v6.o</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>rt_memcpy_v6.o</c:v>
+                  <c:v>init_alloc.o</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>init_alloc.o</c:v>
+                  <c:v>strcmpv7em.o</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>strcmpv7em.o</c:v>
+                  <c:v>llsdiv.o</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>_printf_dec.o</c:v>
+                  <c:v>rt_memcpy_w.o</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>llsdiv.o</c:v>
+                  <c:v>h1_alloc.o</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>__printf.o</c:v>
+                  <c:v>__scatter.o</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>rt_memcpy_w.o</c:v>
+                  <c:v>defsig_rtmem_inner.o</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>h1_alloc.o</c:v>
+                  <c:v>rt_memclr_w.o</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>__scatter.o</c:v>
+                  <c:v>h1_free.o</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>defsig_rtmem_inner.o</c:v>
+                  <c:v>fclose.o</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>rt_memclr_w.o</c:v>
+                  <c:v>sys_stackheap_outer.o</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>h1_free.o</c:v>
+                  <c:v>strcpy.o</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>fclose.o</c:v>
+                  <c:v>setvbuf.o</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>sys_stackheap_outer.o</c:v>
+                  <c:v>rt_memclr.o</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>strcpy.o</c:v>
+                  <c:v>ftell.o</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>setvbuf.o</c:v>
+                  <c:v>strlen.o</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>rt_memclr.o</c:v>
+                  <c:v>h1_extend.o</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>ftell.o</c:v>
+                  <c:v>defsig_rtred_inner.o</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>strlen.o</c:v>
+                  <c:v>defsig_general.o</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>h1_extend.o</c:v>
+                  <c:v>puts.o</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>defsig_rtred_inner.o</c:v>
+                  <c:v>init_aeabi.o</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>defsig_general.o</c:v>
+                  <c:v>systick_wrapper_gnu.o</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>_printf_char_common.o</c:v>
+                  <c:v>fputc.o</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>puts.o</c:v>
+                  <c:v>__scatter_zi.o</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>init_aeabi.o</c:v>
+                  <c:v>fz_wm.l</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>_printf_char_file.o</c:v>
+                  <c:v>fpinit.o</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>systick_wrapper_gnu.o</c:v>
+                  <c:v>__scatter_copy.o</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>fputc.o</c:v>
+                  <c:v>libinit2.o</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>__scatter_zi.o</c:v>
+                  <c:v>exit.o</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>fz_wm.l</c:v>
+                  <c:v>aeabi_memset4.o</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>fpinit.o</c:v>
+                  <c:v>aeabi_memset.o</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>__scatter_copy.o</c:v>
+                  <c:v>sys_wrch.o</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>noretval__2printf.o</c:v>
+                  <c:v>defsig_rtred_outer.o</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>libinit2.o</c:v>
+                  <c:v>defsig_rtmem_outer.o</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>exit.o</c:v>
+                  <c:v>sys_exit.o</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>aeabi_memset4.o</c:v>
+                  <c:v>stdio_streams.o</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>aeabi_memset.o</c:v>
+                  <c:v>h1_init.o</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>sys_wrch.o</c:v>
+                  <c:v>__rtentry2.o</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>defsig_rtred_outer.o</c:v>
+                  <c:v>rtexit2.o</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>defsig_rtmem_outer.o</c:v>
+                  <c:v>defsig_exit.o</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>sys_exit.o</c:v>
+                  <c:v>rt_errno_addr_intlibspace.o</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>stdio_streams.o</c:v>
+                  <c:v>libspace.o</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>h1_init.o</c:v>
+                  <c:v>__main.o</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>__rtentry2.o</c:v>
+                  <c:v>libshutdown2.o</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>rtexit2.o</c:v>
+                  <c:v>heapauxi.o</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>defsig_exit.o</c:v>
+                  <c:v>__rtentry4.o</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>rt_errno_addr_intlibspace.o</c:v>
+                  <c:v>hguard.o</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>libspace.o</c:v>
+                  <c:v>use_no_semi.o</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>ferror.o</c:v>
+                  <c:v>rtexit.o</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>__main.o</c:v>
+                  <c:v>libshutdown.o</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>libshutdown2.o</c:v>
+                  <c:v>libinit.o</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>heapauxi.o</c:v>
-                </c:pt>
-                <c:pt idx="62">
-                  <c:v>_printf_u.o</c:v>
-                </c:pt>
-                <c:pt idx="63">
-                  <c:v>__rtentry4.o</c:v>
-                </c:pt>
-                <c:pt idx="64">
-                  <c:v>hguard.o</c:v>
-                </c:pt>
-                <c:pt idx="65">
-                  <c:v>_printf_percent_end.o</c:v>
-                </c:pt>
-                <c:pt idx="66">
-                  <c:v>use_no_semi.o</c:v>
-                </c:pt>
-                <c:pt idx="67">
-                  <c:v>rtexit.o</c:v>
-                </c:pt>
-                <c:pt idx="68">
-                  <c:v>libshutdown.o</c:v>
-                </c:pt>
-                <c:pt idx="69">
-                  <c:v>libinit.o</c:v>
-                </c:pt>
-                <c:pt idx="70">
                   <c:v>Totals</c:v>
                 </c:pt>
               </c:strCache>
@@ -681,221 +627,194 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>flash_percent!$B$3:$B$73</c:f>
+              <c:f>flash_percent!$B$3:$B$64</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="71"/>
+                <c:ptCount val="62"/>
                 <c:pt idx="0">
-                  <c:v>97.50539398193359</c:v>
+                  <c:v>97.78083801269531</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.176853656768799</c:v>
+                  <c:v>1.038926243782044</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.1286266297101975</c:v>
+                  <c:v>0.1289959996938705</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.1206208243966103</c:v>
+                  <c:v>0.1209672018885613</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.08326039463281632</c:v>
+                  <c:v>0.0834994837641716</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.07045110315084457</c:v>
+                  <c:v>0.07065340876579285</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.06618133932352066</c:v>
+                  <c:v>0.06637138873338699</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.0640464574098587</c:v>
+                  <c:v>0.06423037499189377</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.0640464574098587</c:v>
+                  <c:v>0.06423037499189377</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.04750112071633339</c:v>
+                  <c:v>0.03693246468901634</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.03682671114802361</c:v>
+                  <c:v>0.03693246468901634</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.03682671114802361</c:v>
+                  <c:v>0.0331856943666935</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.03309066966176033</c:v>
+                  <c:v>0.03104468062520027</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.03202322870492935</c:v>
+                  <c:v>0.02676265500485897</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.03095578588545322</c:v>
+                  <c:v>0.0251568965613842</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.02775346301496029</c:v>
+                  <c:v>0.0251568965613842</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.02668602205812931</c:v>
+                  <c:v>0.02141012437641621</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.02508486062288284</c:v>
+                  <c:v>0.0208748709410429</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.02508486062288284</c:v>
+                  <c:v>0.0208748709410429</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.02134881913661957</c:v>
+                  <c:v>0.02033961750566959</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.02081509865820408</c:v>
+                  <c:v>0.01980436407029629</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.02081509865820408</c:v>
+                  <c:v>0.01926911249756813</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.02028137817978859</c:v>
+                  <c:v>0.01873385906219482</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.0197476577013731</c:v>
+                  <c:v>0.01819860562682152</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.01921393722295761</c:v>
+                  <c:v>0.01766335219144821</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.01868021674454212</c:v>
+                  <c:v>0.01659284718334675</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.01814649626612663</c:v>
+                  <c:v>0.01391658093780279</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.01761277578771114</c:v>
+                  <c:v>0.01391658093780279</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.01654533483088017</c:v>
+                  <c:v>0.01338132750242949</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.01387673150748015</c:v>
+                  <c:v>0.01177556812763214</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.01387673150748015</c:v>
+                  <c:v>0.01177556812763214</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.01334301102906466</c:v>
+                  <c:v>0.008564049378037453</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.01280929055064917</c:v>
+                  <c:v>0.007493543438613415</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>0.01174185052514076</c:v>
+                  <c:v>0.007493543438613415</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>0.01174185052514076</c:v>
+                  <c:v>0.006958290468901396</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>0.009606968611478806</c:v>
+                  <c:v>0.006958290468901396</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>0.008539527654647827</c:v>
+                  <c:v>0.006958290468901396</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>0.007472086232155561</c:v>
+                  <c:v>0.005887784063816071</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>0.007472086232155561</c:v>
+                  <c:v>0.004817278124392033</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>0.006938365753740072</c:v>
+                  <c:v>0.004282024689018726</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>0.006938365753740072</c:v>
+                  <c:v>0.004282024689018726</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>0.006938365753740072</c:v>
+                  <c:v>0.003746771719306707</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>0.006404645275324583</c:v>
+                  <c:v>0.003746771719306707</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>0.005870925262570381</c:v>
+                  <c:v>0.003746771719306707</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>0.004803484305739403</c:v>
+                  <c:v>0.003211518749594688</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>0.004269763827323914</c:v>
+                  <c:v>0.003211518749594688</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>0.004269763827323914</c:v>
+                  <c:v>0.003211518749594688</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>0.003736043116077781</c:v>
+                  <c:v>0.003211518749594688</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>0.003736043116077781</c:v>
+                  <c:v>0.002676265547052026</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>0.003736043116077781</c:v>
+                  <c:v>0.002676265547052026</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>0.003202322637662292</c:v>
+                  <c:v>0.002141012344509363</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>0.003202322637662292</c:v>
+                  <c:v>0.002141012344509363</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>0.003202322637662292</c:v>
+                  <c:v>0.002141012344509363</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>0.003202322637662292</c:v>
+                  <c:v>0.001605759374797344</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>0.002668602392077446</c:v>
+                  <c:v>0.001605759374797344</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>0.002668602392077446</c:v>
+                  <c:v>0.001605759374797344</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>0.002134881913661957</c:v>
+                  <c:v>0.001070506172254682</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>0.002134881913661957</c:v>
+                  <c:v>0.0005352530861273408</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>0.002134881913661957</c:v>
+                  <c:v>0.0005352530861273408</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>0.002134881913661957</c:v>
+                  <c:v>0.0005352530861273408</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>0.001601161318831146</c:v>
+                  <c:v>0.0005352530861273408</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>0.001601161318831146</c:v>
-                </c:pt>
-                <c:pt idx="62">
-                  <c:v>0.001601161318831146</c:v>
-                </c:pt>
-                <c:pt idx="63">
-                  <c:v>0.001601161318831146</c:v>
-                </c:pt>
-                <c:pt idx="64">
-                  <c:v>0.001067440956830978</c:v>
-                </c:pt>
-                <c:pt idx="65">
-                  <c:v>0.001067440956830978</c:v>
-                </c:pt>
-                <c:pt idx="66">
-                  <c:v>0.0005337204784154892</c:v>
-                </c:pt>
-                <c:pt idx="67">
-                  <c:v>0.0005337204784154892</c:v>
-                </c:pt>
-                <c:pt idx="68">
-                  <c:v>0.0005337204784154892</c:v>
-                </c:pt>
-                <c:pt idx="69">
-                  <c:v>0.0005337204784154892</c:v>
-                </c:pt>
-                <c:pt idx="70">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -1000,8 +919,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A2:H73" totalsRowCount="1">
-  <autoFilter ref="A2:H72"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A2:H64" totalsRowCount="1">
+  <autoFilter ref="A2:H63"/>
   <tableColumns count="8">
     <tableColumn id="1" name="File_name" totalsRowLabel="Totals"/>
     <tableColumn id="2" name="ram_percent" totalsRowFunction="sum"/>
@@ -1017,8 +936,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A2:H73" totalsRowCount="1">
-  <autoFilter ref="A2:H72"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A2:H64" totalsRowCount="1">
+  <autoFilter ref="A2:H63"/>
   <tableColumns count="8">
     <tableColumn id="1" name="File_name" totalsRowLabel="Totals"/>
     <tableColumn id="2" name="flash_percent" totalsRowFunction="sum"/>
@@ -1318,7 +1237,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="16.7109375" customWidth="1"/>
@@ -1331,28 +1250,28 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="C2" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="D2" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="E2" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="F2" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="G2" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="H2" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1360,22 +1279,22 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>98.32932281494141</v>
+        <v>98.3292236328125</v>
       </c>
       <c r="C3" s="1">
-        <v>132779</v>
+        <v>132771</v>
       </c>
       <c r="D3" s="1">
-        <v>365380</v>
+        <v>365363</v>
       </c>
       <c r="E3" s="1">
-        <v>347578</v>
+        <v>347640</v>
       </c>
       <c r="F3" s="1">
-        <v>17744</v>
+        <v>17673</v>
       </c>
       <c r="G3" s="1">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="H3" s="1">
         <v>132721</v>
@@ -1386,7 +1305,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2">
-        <v>1.137482881546021</v>
+        <v>1.137550234794617</v>
       </c>
       <c r="C4" s="1">
         <v>1536</v>
@@ -1412,16 +1331,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="2">
-        <v>0.2665975391864777</v>
+        <v>0.2666133344173431</v>
       </c>
       <c r="C5" s="1">
         <v>360</v>
       </c>
       <c r="D5" s="1">
-        <v>4410</v>
+        <v>3882</v>
       </c>
       <c r="E5" s="1">
-        <v>4398</v>
+        <v>3870</v>
       </c>
       <c r="F5" s="1">
         <v>0</v>
@@ -1438,7 +1357,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>0.1955048739910126</v>
+        <v>0.1955164521932602</v>
       </c>
       <c r="C6" s="1">
         <v>264</v>
@@ -1464,7 +1383,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>0.07109268009662628</v>
+        <v>0.07109688967466354</v>
       </c>
       <c r="C7" s="1">
         <v>96</v>
@@ -1485,35 +1404,35 @@
         <v>96</v>
       </c>
     </row>
-    <row r="73" spans="1:8">
-      <c r="A73" t="s">
-        <v>72</v>
-      </c>
-      <c r="B73">
+    <row r="64" spans="1:8">
+      <c r="A64" t="s">
+        <v>63</v>
+      </c>
+      <c r="B64">
         <f>SUBTOTAL(109,[ram_percent])</f>
         <v>0</v>
       </c>
-      <c r="C73">
+      <c r="C64">
         <f>SUBTOTAL(109,[ram])</f>
         <v>0</v>
       </c>
-      <c r="D73">
+      <c r="D64">
         <f>SUBTOTAL(109,[flash])</f>
         <v>0</v>
       </c>
-      <c r="E73">
+      <c r="E64">
         <f>SUBTOTAL(109,[Code])</f>
         <v>0</v>
       </c>
-      <c r="F73">
+      <c r="F64">
         <f>SUBTOTAL(109,[RO_data])</f>
         <v>0</v>
       </c>
-      <c r="G73">
+      <c r="G64">
         <f>SUBTOTAL(109,[RW_data])</f>
         <v>0</v>
       </c>
-      <c r="H73">
+      <c r="H64">
         <f>SUBTOTAL(109,[ZI_data])</f>
         <v>0</v>
       </c>
@@ -1529,7 +1448,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="16.7109375" customWidth="1"/>
@@ -1542,28 +1461,28 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" t="s">
         <v>71</v>
       </c>
-      <c r="B2" t="s">
-        <v>80</v>
-      </c>
       <c r="C2" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="D2" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="E2" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="F2" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="G2" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="H2" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1571,22 +1490,22 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>97.50539398193359</v>
+        <v>97.78083801269531</v>
       </c>
       <c r="C3" s="1">
-        <v>365380</v>
+        <v>365363</v>
       </c>
       <c r="D3" s="1">
-        <v>132779</v>
+        <v>132771</v>
       </c>
       <c r="E3" s="1">
-        <v>347578</v>
+        <v>347640</v>
       </c>
       <c r="F3" s="1">
-        <v>17744</v>
+        <v>17673</v>
       </c>
       <c r="G3" s="1">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="H3" s="1">
         <v>132721</v>
@@ -1597,16 +1516,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>1.176853656768799</v>
+        <v>1.038926243782044</v>
       </c>
       <c r="C4" s="1">
-        <v>4410</v>
+        <v>3882</v>
       </c>
       <c r="D4" s="1">
         <v>360</v>
       </c>
       <c r="E4" s="1">
-        <v>4398</v>
+        <v>3870</v>
       </c>
       <c r="F4" s="1">
         <v>0</v>
@@ -1623,7 +1542,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="2">
-        <v>0.1286266297101975</v>
+        <v>0.1289959996938705</v>
       </c>
       <c r="C5" s="1">
         <v>482</v>
@@ -1649,7 +1568,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="2">
-        <v>0.1206208243966103</v>
+        <v>0.1209672018885613</v>
       </c>
       <c r="C6" s="1">
         <v>452</v>
@@ -1675,7 +1594,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="2">
-        <v>0.08326039463281632</v>
+        <v>0.0834994837641716</v>
       </c>
       <c r="C7" s="1">
         <v>312</v>
@@ -1701,7 +1620,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="2">
-        <v>0.07045110315084457</v>
+        <v>0.07065340876579285</v>
       </c>
       <c r="C8" s="1">
         <v>264</v>
@@ -1727,7 +1646,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="2">
-        <v>0.06618133932352066</v>
+        <v>0.06637138873338699</v>
       </c>
       <c r="C9" s="1">
         <v>248</v>
@@ -1753,7 +1672,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="2">
-        <v>0.0640464574098587</v>
+        <v>0.06423037499189377</v>
       </c>
       <c r="C10" s="1">
         <v>240</v>
@@ -1779,7 +1698,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="2">
-        <v>0.0640464574098587</v>
+        <v>0.06423037499189377</v>
       </c>
       <c r="C11" s="1">
         <v>240</v>
@@ -1805,16 +1724,16 @@
         <v>12</v>
       </c>
       <c r="B12" s="2">
-        <v>0.04750112071633339</v>
+        <v>0.03693246468901634</v>
       </c>
       <c r="C12" s="1">
-        <v>178</v>
+        <v>138</v>
       </c>
       <c r="D12" s="1">
         <v>0</v>
       </c>
       <c r="E12" s="1">
-        <v>178</v>
+        <v>138</v>
       </c>
       <c r="F12" s="1">
         <v>0</v>
@@ -1831,7 +1750,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="2">
-        <v>0.03682671114802361</v>
+        <v>0.03693246468901634</v>
       </c>
       <c r="C13" s="1">
         <v>138</v>
@@ -1857,16 +1776,16 @@
         <v>14</v>
       </c>
       <c r="B14" s="2">
-        <v>0.03682671114802361</v>
+        <v>0.0331856943666935</v>
       </c>
       <c r="C14" s="1">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="D14" s="1">
         <v>0</v>
       </c>
       <c r="E14" s="1">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="F14" s="1">
         <v>0</v>
@@ -1883,16 +1802,16 @@
         <v>15</v>
       </c>
       <c r="B15" s="2">
-        <v>0.03309066966176033</v>
+        <v>0.03104468062520027</v>
       </c>
       <c r="C15" s="1">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="D15" s="1">
         <v>0</v>
       </c>
       <c r="E15" s="1">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="F15" s="1">
         <v>0</v>
@@ -1909,16 +1828,16 @@
         <v>16</v>
       </c>
       <c r="B16" s="2">
-        <v>0.03202322870492935</v>
+        <v>0.02676265500485897</v>
       </c>
       <c r="C16" s="1">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D16" s="1">
         <v>0</v>
       </c>
       <c r="E16" s="1">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="F16" s="1">
         <v>0</v>
@@ -1935,16 +1854,16 @@
         <v>17</v>
       </c>
       <c r="B17" s="2">
-        <v>0.03095578588545322</v>
+        <v>0.0251568965613842</v>
       </c>
       <c r="C17" s="1">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="D17" s="1">
         <v>0</v>
       </c>
       <c r="E17" s="1">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="F17" s="1">
         <v>0</v>
@@ -1961,16 +1880,16 @@
         <v>18</v>
       </c>
       <c r="B18" s="2">
-        <v>0.02775346301496029</v>
+        <v>0.0251568965613842</v>
       </c>
       <c r="C18" s="1">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="D18" s="1">
         <v>0</v>
       </c>
       <c r="E18" s="1">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="F18" s="1">
         <v>0</v>
@@ -1987,16 +1906,16 @@
         <v>19</v>
       </c>
       <c r="B19" s="2">
-        <v>0.02668602205812931</v>
+        <v>0.02141012437641621</v>
       </c>
       <c r="C19" s="1">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="D19" s="1">
         <v>0</v>
       </c>
       <c r="E19" s="1">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="F19" s="1">
         <v>0</v>
@@ -2013,16 +1932,16 @@
         <v>20</v>
       </c>
       <c r="B20" s="2">
-        <v>0.02508486062288284</v>
+        <v>0.0208748709410429</v>
       </c>
       <c r="C20" s="1">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="D20" s="1">
         <v>0</v>
       </c>
       <c r="E20" s="1">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="F20" s="1">
         <v>0</v>
@@ -2039,16 +1958,16 @@
         <v>21</v>
       </c>
       <c r="B21" s="2">
-        <v>0.02508486062288284</v>
+        <v>0.0208748709410429</v>
       </c>
       <c r="C21" s="1">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="D21" s="1">
         <v>0</v>
       </c>
       <c r="E21" s="1">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="F21" s="1">
         <v>0</v>
@@ -2065,16 +1984,16 @@
         <v>22</v>
       </c>
       <c r="B22" s="2">
-        <v>0.02134881913661957</v>
+        <v>0.02033961750566959</v>
       </c>
       <c r="C22" s="1">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D22" s="1">
         <v>0</v>
       </c>
       <c r="E22" s="1">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F22" s="1">
         <v>0</v>
@@ -2091,16 +2010,16 @@
         <v>23</v>
       </c>
       <c r="B23" s="2">
-        <v>0.02081509865820408</v>
+        <v>0.01980436407029629</v>
       </c>
       <c r="C23" s="1">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D23" s="1">
         <v>0</v>
       </c>
       <c r="E23" s="1">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F23" s="1">
         <v>0</v>
@@ -2117,16 +2036,16 @@
         <v>24</v>
       </c>
       <c r="B24" s="2">
-        <v>0.02081509865820408</v>
+        <v>0.01926911249756813</v>
       </c>
       <c r="C24" s="1">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="D24" s="1">
         <v>0</v>
       </c>
       <c r="E24" s="1">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="F24" s="1">
         <v>0</v>
@@ -2143,16 +2062,16 @@
         <v>25</v>
       </c>
       <c r="B25" s="2">
-        <v>0.02028137817978859</v>
+        <v>0.01873385906219482</v>
       </c>
       <c r="C25" s="1">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="D25" s="1">
         <v>0</v>
       </c>
       <c r="E25" s="1">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="F25" s="1">
         <v>0</v>
@@ -2169,16 +2088,16 @@
         <v>26</v>
       </c>
       <c r="B26" s="2">
-        <v>0.0197476577013731</v>
+        <v>0.01819860562682152</v>
       </c>
       <c r="C26" s="1">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D26" s="1">
         <v>0</v>
       </c>
       <c r="E26" s="1">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F26" s="1">
         <v>0</v>
@@ -2195,16 +2114,16 @@
         <v>27</v>
       </c>
       <c r="B27" s="2">
-        <v>0.01921393722295761</v>
+        <v>0.01766335219144821</v>
       </c>
       <c r="C27" s="1">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D27" s="1">
         <v>0</v>
       </c>
       <c r="E27" s="1">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="F27" s="1">
         <v>0</v>
@@ -2221,16 +2140,16 @@
         <v>28</v>
       </c>
       <c r="B28" s="2">
-        <v>0.01868021674454212</v>
+        <v>0.01659284718334675</v>
       </c>
       <c r="C28" s="1">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="D28" s="1">
         <v>0</v>
       </c>
       <c r="E28" s="1">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="F28" s="1">
         <v>0</v>
@@ -2247,16 +2166,16 @@
         <v>29</v>
       </c>
       <c r="B29" s="2">
-        <v>0.01814649626612663</v>
+        <v>0.01391658093780279</v>
       </c>
       <c r="C29" s="1">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="D29" s="1">
         <v>0</v>
       </c>
       <c r="E29" s="1">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="F29" s="1">
         <v>0</v>
@@ -2273,16 +2192,16 @@
         <v>30</v>
       </c>
       <c r="B30" s="2">
-        <v>0.01761277578771114</v>
+        <v>0.01391658093780279</v>
       </c>
       <c r="C30" s="1">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="D30" s="1">
         <v>0</v>
       </c>
       <c r="E30" s="1">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="F30" s="1">
         <v>0</v>
@@ -2299,16 +2218,16 @@
         <v>31</v>
       </c>
       <c r="B31" s="2">
-        <v>0.01654533483088017</v>
+        <v>0.01338132750242949</v>
       </c>
       <c r="C31" s="1">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="D31" s="1">
         <v>0</v>
       </c>
       <c r="E31" s="1">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="F31" s="1">
         <v>0</v>
@@ -2325,16 +2244,16 @@
         <v>32</v>
       </c>
       <c r="B32" s="2">
-        <v>0.01387673150748015</v>
+        <v>0.01177556812763214</v>
       </c>
       <c r="C32" s="1">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="D32" s="1">
         <v>0</v>
       </c>
       <c r="E32" s="1">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="F32" s="1">
         <v>0</v>
@@ -2351,16 +2270,16 @@
         <v>33</v>
       </c>
       <c r="B33" s="2">
-        <v>0.01387673150748015</v>
+        <v>0.01177556812763214</v>
       </c>
       <c r="C33" s="1">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="D33" s="1">
         <v>0</v>
       </c>
       <c r="E33" s="1">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="F33" s="1">
         <v>0</v>
@@ -2377,16 +2296,16 @@
         <v>34</v>
       </c>
       <c r="B34" s="2">
-        <v>0.01334301102906466</v>
+        <v>0.008564049378037453</v>
       </c>
       <c r="C34" s="1">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="D34" s="1">
         <v>0</v>
       </c>
       <c r="E34" s="1">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="F34" s="1">
         <v>0</v>
@@ -2403,16 +2322,16 @@
         <v>35</v>
       </c>
       <c r="B35" s="2">
-        <v>0.01280929055064917</v>
+        <v>0.007493543438613415</v>
       </c>
       <c r="C35" s="1">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="D35" s="1">
         <v>0</v>
       </c>
       <c r="E35" s="1">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="F35" s="1">
         <v>0</v>
@@ -2429,16 +2348,16 @@
         <v>36</v>
       </c>
       <c r="B36" s="2">
-        <v>0.01174185052514076</v>
+        <v>0.007493543438613415</v>
       </c>
       <c r="C36" s="1">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="D36" s="1">
         <v>0</v>
       </c>
       <c r="E36" s="1">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="F36" s="1">
         <v>0</v>
@@ -2455,16 +2374,16 @@
         <v>37</v>
       </c>
       <c r="B37" s="2">
-        <v>0.01174185052514076</v>
+        <v>0.006958290468901396</v>
       </c>
       <c r="C37" s="1">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="D37" s="1">
         <v>0</v>
       </c>
       <c r="E37" s="1">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="F37" s="1">
         <v>0</v>
@@ -2481,16 +2400,16 @@
         <v>38</v>
       </c>
       <c r="B38" s="2">
-        <v>0.009606968611478806</v>
+        <v>0.006958290468901396</v>
       </c>
       <c r="C38" s="1">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="D38" s="1">
         <v>0</v>
       </c>
       <c r="E38" s="1">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="F38" s="1">
         <v>0</v>
@@ -2507,16 +2426,16 @@
         <v>39</v>
       </c>
       <c r="B39" s="2">
-        <v>0.008539527654647827</v>
+        <v>0.006958290468901396</v>
       </c>
       <c r="C39" s="1">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D39" s="1">
         <v>0</v>
       </c>
       <c r="E39" s="1">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F39" s="1">
         <v>0</v>
@@ -2533,16 +2452,16 @@
         <v>40</v>
       </c>
       <c r="B40" s="2">
-        <v>0.007472086232155561</v>
+        <v>0.005887784063816071</v>
       </c>
       <c r="C40" s="1">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="D40" s="1">
         <v>0</v>
       </c>
       <c r="E40" s="1">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="F40" s="1">
         <v>0</v>
@@ -2559,16 +2478,16 @@
         <v>41</v>
       </c>
       <c r="B41" s="2">
-        <v>0.007472086232155561</v>
+        <v>0.004817278124392033</v>
       </c>
       <c r="C41" s="1">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="D41" s="1">
         <v>0</v>
       </c>
       <c r="E41" s="1">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F41" s="1">
         <v>0</v>
@@ -2585,16 +2504,16 @@
         <v>42</v>
       </c>
       <c r="B42" s="2">
-        <v>0.006938365753740072</v>
+        <v>0.004282024689018726</v>
       </c>
       <c r="C42" s="1">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="D42" s="1">
         <v>0</v>
       </c>
       <c r="E42" s="1">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F42" s="1">
         <v>0</v>
@@ -2611,16 +2530,16 @@
         <v>43</v>
       </c>
       <c r="B43" s="2">
-        <v>0.006938365753740072</v>
+        <v>0.004282024689018726</v>
       </c>
       <c r="C43" s="1">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="D43" s="1">
         <v>0</v>
       </c>
       <c r="E43" s="1">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F43" s="1">
         <v>0</v>
@@ -2637,16 +2556,16 @@
         <v>44</v>
       </c>
       <c r="B44" s="2">
-        <v>0.006938365753740072</v>
+        <v>0.003746771719306707</v>
       </c>
       <c r="C44" s="1">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="D44" s="1">
         <v>0</v>
       </c>
       <c r="E44" s="1">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="F44" s="1">
         <v>0</v>
@@ -2663,16 +2582,16 @@
         <v>45</v>
       </c>
       <c r="B45" s="2">
-        <v>0.006404645275324583</v>
+        <v>0.003746771719306707</v>
       </c>
       <c r="C45" s="1">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D45" s="1">
         <v>0</v>
       </c>
       <c r="E45" s="1">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F45" s="1">
         <v>0</v>
@@ -2689,16 +2608,16 @@
         <v>46</v>
       </c>
       <c r="B46" s="2">
-        <v>0.005870925262570381</v>
+        <v>0.003746771719306707</v>
       </c>
       <c r="C46" s="1">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D46" s="1">
         <v>0</v>
       </c>
       <c r="E46" s="1">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F46" s="1">
         <v>0</v>
@@ -2715,16 +2634,16 @@
         <v>47</v>
       </c>
       <c r="B47" s="2">
-        <v>0.004803484305739403</v>
+        <v>0.003211518749594688</v>
       </c>
       <c r="C47" s="1">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D47" s="1">
         <v>0</v>
       </c>
       <c r="E47" s="1">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F47" s="1">
         <v>0</v>
@@ -2738,45 +2657,45 @@
     </row>
     <row r="48" spans="1:8">
       <c r="A48" s="1" t="s">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="B48" s="2">
-        <v>0.004269763827323914</v>
+        <v>0.003211518749594688</v>
       </c>
       <c r="C48" s="1">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D48" s="1">
-        <v>0</v>
+        <v>264</v>
       </c>
       <c r="E48" s="1">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="F48" s="1">
         <v>0</v>
       </c>
       <c r="G48" s="1">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H48" s="1">
-        <v>0</v>
+        <v>252</v>
       </c>
     </row>
     <row r="49" spans="1:8">
       <c r="A49" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B49" s="2">
-        <v>0.004269763827323914</v>
+        <v>0.003211518749594688</v>
       </c>
       <c r="C49" s="1">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D49" s="1">
         <v>0</v>
       </c>
       <c r="E49" s="1">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F49" s="1">
         <v>0</v>
@@ -2790,19 +2709,19 @@
     </row>
     <row r="50" spans="1:8">
       <c r="A50" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B50" s="2">
-        <v>0.003736043116077781</v>
+        <v>0.003211518749594688</v>
       </c>
       <c r="C50" s="1">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D50" s="1">
         <v>0</v>
       </c>
       <c r="E50" s="1">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F50" s="1">
         <v>0</v>
@@ -2816,19 +2735,19 @@
     </row>
     <row r="51" spans="1:8">
       <c r="A51" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B51" s="2">
-        <v>0.003736043116077781</v>
+        <v>0.002676265547052026</v>
       </c>
       <c r="C51" s="1">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D51" s="1">
         <v>0</v>
       </c>
       <c r="E51" s="1">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F51" s="1">
         <v>0</v>
@@ -2842,19 +2761,19 @@
     </row>
     <row r="52" spans="1:8">
       <c r="A52" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B52" s="2">
-        <v>0.003736043116077781</v>
+        <v>0.002676265547052026</v>
       </c>
       <c r="C52" s="1">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D52" s="1">
         <v>0</v>
       </c>
       <c r="E52" s="1">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F52" s="1">
         <v>0</v>
@@ -2868,19 +2787,19 @@
     </row>
     <row r="53" spans="1:8">
       <c r="A53" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B53" s="2">
-        <v>0.003202322637662292</v>
+        <v>0.002141012344509363</v>
       </c>
       <c r="C53" s="1">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D53" s="1">
         <v>0</v>
       </c>
       <c r="E53" s="1">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F53" s="1">
         <v>0</v>
@@ -2894,45 +2813,45 @@
     </row>
     <row r="54" spans="1:8">
       <c r="A54" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B54" s="2">
-        <v>0.003202322637662292</v>
+        <v>0.002141012344509363</v>
       </c>
       <c r="C54" s="1">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D54" s="1">
-        <v>264</v>
+        <v>96</v>
       </c>
       <c r="E54" s="1">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F54" s="1">
         <v>0</v>
       </c>
       <c r="G54" s="1">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H54" s="1">
-        <v>252</v>
+        <v>96</v>
       </c>
     </row>
     <row r="55" spans="1:8">
       <c r="A55" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B55" s="2">
-        <v>0.003202322637662292</v>
+        <v>0.002141012344509363</v>
       </c>
       <c r="C55" s="1">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D55" s="1">
         <v>0</v>
       </c>
       <c r="E55" s="1">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F55" s="1">
         <v>0</v>
@@ -2946,19 +2865,19 @@
     </row>
     <row r="56" spans="1:8">
       <c r="A56" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B56" s="2">
-        <v>0.003202322637662292</v>
+        <v>0.001605759374797344</v>
       </c>
       <c r="C56" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D56" s="1">
         <v>0</v>
       </c>
       <c r="E56" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F56" s="1">
         <v>0</v>
@@ -2972,19 +2891,19 @@
     </row>
     <row r="57" spans="1:8">
       <c r="A57" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B57" s="2">
-        <v>0.002668602392077446</v>
+        <v>0.001605759374797344</v>
       </c>
       <c r="C57" s="1">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D57" s="1">
         <v>0</v>
       </c>
       <c r="E57" s="1">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F57" s="1">
         <v>0</v>
@@ -2998,19 +2917,19 @@
     </row>
     <row r="58" spans="1:8">
       <c r="A58" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B58" s="2">
-        <v>0.002668602392077446</v>
+        <v>0.001605759374797344</v>
       </c>
       <c r="C58" s="1">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D58" s="1">
         <v>0</v>
       </c>
       <c r="E58" s="1">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F58" s="1">
         <v>0</v>
@@ -3024,19 +2943,19 @@
     </row>
     <row r="59" spans="1:8">
       <c r="A59" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B59" s="2">
-        <v>0.002134881913661957</v>
+        <v>0.001070506172254682</v>
       </c>
       <c r="C59" s="1">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D59" s="1">
         <v>0</v>
       </c>
       <c r="E59" s="1">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F59" s="1">
         <v>0</v>
@@ -3050,19 +2969,19 @@
     </row>
     <row r="60" spans="1:8">
       <c r="A60" s="1" t="s">
-        <v>5</v>
+        <v>58</v>
       </c>
       <c r="B60" s="2">
-        <v>0.002134881913661957</v>
+        <v>0.0005352530861273408</v>
       </c>
       <c r="C60" s="1">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D60" s="1">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="E60" s="1">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F60" s="1">
         <v>0</v>
@@ -3071,7 +2990,7 @@
         <v>0</v>
       </c>
       <c r="H60" s="1">
-        <v>96</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61" spans="1:8">
@@ -3079,16 +2998,16 @@
         <v>59</v>
       </c>
       <c r="B61" s="2">
-        <v>0.002134881913661957</v>
+        <v>0.0005352530861273408</v>
       </c>
       <c r="C61" s="1">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D61" s="1">
         <v>0</v>
       </c>
       <c r="E61" s="1">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F61" s="1">
         <v>0</v>
@@ -3105,16 +3024,16 @@
         <v>60</v>
       </c>
       <c r="B62" s="2">
-        <v>0.002134881913661957</v>
+        <v>0.0005352530861273408</v>
       </c>
       <c r="C62" s="1">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D62" s="1">
         <v>0</v>
       </c>
       <c r="E62" s="1">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F62" s="1">
         <v>0</v>
@@ -3131,16 +3050,16 @@
         <v>61</v>
       </c>
       <c r="B63" s="2">
-        <v>0.001601161318831146</v>
+        <v>0.0005352530861273408</v>
       </c>
       <c r="C63" s="1">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D63" s="1">
         <v>0</v>
       </c>
       <c r="E63" s="1">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F63" s="1">
         <v>0</v>
@@ -3153,268 +3072,34 @@
       </c>
     </row>
     <row r="64" spans="1:8">
-      <c r="A64" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B64" s="2">
-        <v>0.001601161318831146</v>
-      </c>
-      <c r="C64" s="1">
-        <v>6</v>
-      </c>
-      <c r="D64" s="1">
-        <v>0</v>
-      </c>
-      <c r="E64" s="1">
-        <v>6</v>
-      </c>
-      <c r="F64" s="1">
-        <v>0</v>
-      </c>
-      <c r="G64" s="1">
-        <v>0</v>
-      </c>
-      <c r="H64" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:8">
-      <c r="A65" s="1" t="s">
+      <c r="A64" t="s">
         <v>63</v>
       </c>
-      <c r="B65" s="2">
-        <v>0.001601161318831146</v>
-      </c>
-      <c r="C65" s="1">
-        <v>6</v>
-      </c>
-      <c r="D65" s="1">
-        <v>0</v>
-      </c>
-      <c r="E65" s="1">
-        <v>6</v>
-      </c>
-      <c r="F65" s="1">
-        <v>0</v>
-      </c>
-      <c r="G65" s="1">
-        <v>0</v>
-      </c>
-      <c r="H65" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:8">
-      <c r="A66" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B66" s="2">
-        <v>0.001601161318831146</v>
-      </c>
-      <c r="C66" s="1">
-        <v>6</v>
-      </c>
-      <c r="D66" s="1">
-        <v>0</v>
-      </c>
-      <c r="E66" s="1">
-        <v>6</v>
-      </c>
-      <c r="F66" s="1">
-        <v>0</v>
-      </c>
-      <c r="G66" s="1">
-        <v>0</v>
-      </c>
-      <c r="H66" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:8">
-      <c r="A67" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="B67" s="2">
-        <v>0.001067440956830978</v>
-      </c>
-      <c r="C67" s="1">
-        <v>4</v>
-      </c>
-      <c r="D67" s="1">
-        <v>0</v>
-      </c>
-      <c r="E67" s="1">
-        <v>4</v>
-      </c>
-      <c r="F67" s="1">
-        <v>0</v>
-      </c>
-      <c r="G67" s="1">
-        <v>0</v>
-      </c>
-      <c r="H67" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" spans="1:8">
-      <c r="A68" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B68" s="2">
-        <v>0.001067440956830978</v>
-      </c>
-      <c r="C68" s="1">
-        <v>4</v>
-      </c>
-      <c r="D68" s="1">
-        <v>0</v>
-      </c>
-      <c r="E68" s="1">
-        <v>4</v>
-      </c>
-      <c r="F68" s="1">
-        <v>0</v>
-      </c>
-      <c r="G68" s="1">
-        <v>0</v>
-      </c>
-      <c r="H68" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" spans="1:8">
-      <c r="A69" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B69" s="2">
-        <v>0.0005337204784154892</v>
-      </c>
-      <c r="C69" s="1">
-        <v>2</v>
-      </c>
-      <c r="D69" s="1">
-        <v>0</v>
-      </c>
-      <c r="E69" s="1">
-        <v>2</v>
-      </c>
-      <c r="F69" s="1">
-        <v>0</v>
-      </c>
-      <c r="G69" s="1">
-        <v>0</v>
-      </c>
-      <c r="H69" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" spans="1:8">
-      <c r="A70" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B70" s="2">
-        <v>0.0005337204784154892</v>
-      </c>
-      <c r="C70" s="1">
-        <v>2</v>
-      </c>
-      <c r="D70" s="1">
-        <v>0</v>
-      </c>
-      <c r="E70" s="1">
-        <v>2</v>
-      </c>
-      <c r="F70" s="1">
-        <v>0</v>
-      </c>
-      <c r="G70" s="1">
-        <v>0</v>
-      </c>
-      <c r="H70" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="1:8">
-      <c r="A71" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B71" s="2">
-        <v>0.0005337204784154892</v>
-      </c>
-      <c r="C71" s="1">
-        <v>2</v>
-      </c>
-      <c r="D71" s="1">
-        <v>0</v>
-      </c>
-      <c r="E71" s="1">
-        <v>2</v>
-      </c>
-      <c r="F71" s="1">
-        <v>0</v>
-      </c>
-      <c r="G71" s="1">
-        <v>0</v>
-      </c>
-      <c r="H71" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="1:8">
-      <c r="A72" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B72" s="2">
-        <v>0.0005337204784154892</v>
-      </c>
-      <c r="C72" s="1">
-        <v>2</v>
-      </c>
-      <c r="D72" s="1">
-        <v>0</v>
-      </c>
-      <c r="E72" s="1">
-        <v>2</v>
-      </c>
-      <c r="F72" s="1">
-        <v>0</v>
-      </c>
-      <c r="G72" s="1">
-        <v>0</v>
-      </c>
-      <c r="H72" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" spans="1:8">
-      <c r="A73" t="s">
-        <v>72</v>
-      </c>
-      <c r="B73">
+      <c r="B64">
         <f>SUBTOTAL(109,[flash_percent])</f>
         <v>0</v>
       </c>
-      <c r="C73">
+      <c r="C64">
         <f>SUBTOTAL(109,[flash])</f>
         <v>0</v>
       </c>
-      <c r="D73">
+      <c r="D64">
         <f>SUBTOTAL(109,[ram])</f>
         <v>0</v>
       </c>
-      <c r="E73">
+      <c r="E64">
         <f>SUBTOTAL(109,[Code])</f>
         <v>0</v>
       </c>
-      <c r="F73">
+      <c r="F64">
         <f>SUBTOTAL(109,[RO_data])</f>
         <v>0</v>
       </c>
-      <c r="G73">
+      <c r="G64">
         <f>SUBTOTAL(109,[RW_data])</f>
         <v>0</v>
       </c>
-      <c r="H73">
+      <c r="H64">
         <f>SUBTOTAL(109,[ZI_data])</f>
         <v>0</v>
       </c>

</xml_diff>